<commit_message>
Changed files structure added some files
</commit_message>
<xml_diff>
--- a/Zeszyt1.xlsx
+++ b/Zeszyt1.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mati7\ProjektBazyDanych\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615B9233-2583-46EB-8F2E-C7AF11F34836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1257B29A-B2EB-4397-970D-B60522256446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-1800" windowWidth="19440" windowHeight="15000" xr2:uid="{81237377-BF7B-462D-9061-7DD7B93E43FE}"/>
+    <workbookView xWindow="-19320" yWindow="-1800" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{81237377-BF7B-462D-9061-7DD7B93E43FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
+    <sheet name="Features" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Arkusz1!$A$1:$C$1</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="77">
   <si>
     <t>Tabela nadrzędna przechowująca podstawowe dane osób znajdujących się w systemie (pracownicy i klienci), takie jak imię, nazwisko, PESEL, e-mail i miasto.</t>
   </si>
@@ -144,6 +145,132 @@
   </si>
   <si>
     <t>liczba rekordów</t>
+  </si>
+  <si>
+    <t>FunctionsViews.sql</t>
+  </si>
+  <si>
+    <t>Triggers.sql</t>
+  </si>
+  <si>
+    <t>Procedures.sql</t>
+  </si>
+  <si>
+    <t>dbo.GetMonthlyPayouts(INT)</t>
+  </si>
+  <si>
+    <t>function</t>
+  </si>
+  <si>
+    <t>Zwraca wyplate kazdego pracownika za dany miesiac</t>
+  </si>
+  <si>
+    <t>PopularClasses</t>
+  </si>
+  <si>
+    <t>view</t>
+  </si>
+  <si>
+    <t>Zwraca sume wszytskichrejestracji na dany typ zajec</t>
+  </si>
+  <si>
+    <t>dbo.GetAccessPermission(INT,DATE)</t>
+  </si>
+  <si>
+    <t>Zwraca 1 albo 0 w zaleznosci od mozliwosci wejscia na silownie</t>
+  </si>
+  <si>
+    <t>CustomersSpending</t>
+  </si>
+  <si>
+    <t>Zwraca ile każdy nasz klient wydal lacznie pieniedzy</t>
+  </si>
+  <si>
+    <t>TR_UpdateRegisteredCount</t>
+  </si>
+  <si>
+    <t>trigger</t>
+  </si>
+  <si>
+    <t>Aktualizuje liczbe zapisanych osob na zajecia</t>
+  </si>
+  <si>
+    <t>TR_GeneratePaymentForSingleEntry</t>
+  </si>
+  <si>
+    <t>Symuluje wystawienie rachunku za PojedynczeWejscie</t>
+  </si>
+  <si>
+    <t>TR_GeneratePaymentForMembership</t>
+  </si>
+  <si>
+    <t>Symuluje wystawienie rachunku za  Karnet</t>
+  </si>
+  <si>
+    <t>TR_GeneratePaymentForReservations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">trigger </t>
+  </si>
+  <si>
+    <t>Symuluje wystawienie rachunku za  rezerwacje Sali</t>
+  </si>
+  <si>
+    <t>TR_GeneratePaymentForPersonalTrainingSessions</t>
+  </si>
+  <si>
+    <t>Symuluje wystawienie rachunku za  trening</t>
+  </si>
+  <si>
+    <t>dbo.AddCustomer</t>
+  </si>
+  <si>
+    <t>dbo.AddEmployee</t>
+  </si>
+  <si>
+    <t>procedura</t>
+  </si>
+  <si>
+    <t>Dodaje klienta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dodaje pracownika </t>
+  </si>
+  <si>
+    <t>Atrybutem zmieniajacym wartosc w czasie jest Price z [Services]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Po aktualizacji ceny stare rekordy wraz ze stara cena sa utrwalone </t>
+  </si>
+  <si>
+    <t>TestOfTime.sql dowodzi powyzszemu</t>
+  </si>
+  <si>
+    <t>dbo.AddShift</t>
+  </si>
+  <si>
+    <t>Dodaje zmiane</t>
+  </si>
+  <si>
+    <t>dbo.DeleteShift</t>
+  </si>
+  <si>
+    <t>usuwa zmiane</t>
+  </si>
+  <si>
+    <t>dbo.UpdateShift</t>
+  </si>
+  <si>
+    <t>aktualizuje zmiane</t>
+  </si>
+  <si>
+    <t>To wlasnie w ramach WorkShifts będzie udostepniona pelna edycja</t>
+  </si>
+  <si>
+    <t>Photo used in app  https://pixabay.com/photos/weights-gym-dumbbell-gray-gym-3942914/</t>
+  </si>
+  <si>
+    <t>under content license</t>
   </si>
 </sst>
 </file>
@@ -192,10 +319,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -733,4 +866,222 @@
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D6E171-F477-4450-87B1-CAFB5B960CA9}">
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="56.109375" customWidth="1"/>
+    <col min="5" max="5" width="78" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="E7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added function for displaying Classes for the given month and added dbo. prefix
</commit_message>
<xml_diff>
--- a/Zeszyt1.xlsx
+++ b/Zeszyt1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mati7\ProjektBazyDanych\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1257B29A-B2EB-4397-970D-B60522256446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB66A27-8D3B-405D-AE6B-5F3EB26E26DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19320" yWindow="-1800" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{81237377-BF7B-462D-9061-7DD7B93E43FE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
   <si>
     <t>Tabela nadrzędna przechowująca podstawowe dane osób znajdujących się w systemie (pracownicy i klienci), takie jak imię, nazwisko, PESEL, e-mail i miasto.</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>under content license</t>
+  </si>
+  <si>
+    <t>Zwraca grafik na dany miesiac</t>
+  </si>
+  <si>
+    <t>dbo.GetClassSchedule(INT)</t>
   </si>
 </sst>
 </file>
@@ -870,7 +876,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D6E171-F477-4450-87B1-CAFB5B960CA9}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
@@ -942,136 +948,147 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="E7" t="s">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="E8" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
         <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>50</v>
+      </c>
+      <c r="E9" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
         <v>49</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
         <v>56</v>
       </c>
       <c r="C12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>60</v>
-      </c>
-      <c r="B16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" t="s">
-        <v>63</v>
-      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" t="s">
         <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B18" t="s">
         <v>62</v>
       </c>
       <c r="C18" t="s">
-        <v>69</v>
-      </c>
-      <c r="E18" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B19" t="s">
         <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>69</v>
+      </c>
+      <c r="E19" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B20" t="s">
         <v>62</v>
       </c>
       <c r="C20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1079,8 +1096,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed dbo.GetClassSchedule from function to view ( needed for importing whole thing to create a dictionary rather than one month at a time). started working on adding squares to display which class takes place on which day
</commit_message>
<xml_diff>
--- a/Zeszyt1.xlsx
+++ b/Zeszyt1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mati7\ProjektBazyDanych\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB66A27-8D3B-405D-AE6B-5F3EB26E26DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4885934-D7E5-4285-BFD5-0167FC55AE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19320" yWindow="-1800" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{81237377-BF7B-462D-9061-7DD7B93E43FE}"/>
   </bookViews>
@@ -273,10 +273,10 @@
     <t>under content license</t>
   </si>
   <si>
-    <t>Zwraca grafik na dany miesiac</t>
-  </si>
-  <si>
-    <t>dbo.GetClassSchedule(INT)</t>
+    <t>dbo.GetClassSchedule</t>
+  </si>
+  <si>
+    <t>Zwraca caly grafik przygotowany do displayu</t>
   </si>
 </sst>
 </file>
@@ -950,13 +950,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
         <v>78</v>
-      </c>
-      <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Rewrote the App.js code ( got rid of the redundant wrappers and other things which improved responsivity.Added working register button ( only for example user 1 will change after adding logins) added procedure Register for Class
</commit_message>
<xml_diff>
--- a/Zeszyt1.xlsx
+++ b/Zeszyt1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mati7\ProjektBazyDanych\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4885934-D7E5-4285-BFD5-0167FC55AE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD78DA4-3DD5-4E92-8483-E053A112A6D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="-1800" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{81237377-BF7B-462D-9061-7DD7B93E43FE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{81237377-BF7B-462D-9061-7DD7B93E43FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="88">
   <si>
     <t>Tabela nadrzędna przechowująca podstawowe dane osób znajdujących się w systemie (pracownicy i klienci), takie jak imię, nazwisko, PESEL, e-mail i miasto.</t>
   </si>
@@ -277,6 +277,33 @@
   </si>
   <si>
     <t>Zwraca caly grafik przygotowany do displayu</t>
+  </si>
+  <si>
+    <t>dbo.AddClass</t>
+  </si>
+  <si>
+    <t>dbo.DeleteClass</t>
+  </si>
+  <si>
+    <t>dbo.UpdateClass</t>
+  </si>
+  <si>
+    <t>dodaje zajecia</t>
+  </si>
+  <si>
+    <t>usuwa zajecia</t>
+  </si>
+  <si>
+    <t>zmienia dane zajec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">najpierw ClassSchedule jednak </t>
+  </si>
+  <si>
+    <t>dbo.RegisterForClass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rejestruje klienta na zajecia </t>
   </si>
 </sst>
 </file>
@@ -293,7 +320,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -312,6 +339,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -325,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -335,6 +368,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -669,7 +703,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{310DBC49-801B-4EA2-9FA2-F90BF7343E8C}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -759,7 +793,7 @@
         <v>20</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
@@ -781,7 +815,7 @@
         <v>17</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="C10" t="s">
         <v>5</v>
@@ -862,6 +896,12 @@
       </c>
       <c r="C17" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <f>SUM(B2:B17)</f>
+        <v>5600</v>
       </c>
     </row>
   </sheetData>
@@ -876,7 +916,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D6E171-F477-4450-87B1-CAFB5B960CA9}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
@@ -960,144 +1000,209 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="C8" s="5">
+        <f>COUNTA(C2:C6)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="E8" t="s">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="E9" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
         <v>49</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>50</v>
+      </c>
+      <c r="E10" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
         <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
         <v>56</v>
       </c>
       <c r="C13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="C16" s="5">
+        <f>COUNTA(C10:C14)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>60</v>
-      </c>
-      <c r="B17" t="s">
-        <v>62</v>
-      </c>
-      <c r="C17" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" t="s">
-        <v>62</v>
-      </c>
-      <c r="C18" t="s">
-        <v>64</v>
-      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
         <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
         <v>62</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B21" t="s">
         <v>62</v>
       </c>
       <c r="C21" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" t="s">
         <v>73</v>
+      </c>
+      <c r="E23" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>81</v>
+      </c>
+      <c r="B26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>86</v>
+      </c>
+      <c r="B27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C28" s="5">
+        <f>COUNTA(C19:C27)</f>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:F1"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A18:C18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>